<commit_message>
feat(data): add preprocess_nist.py script to extract features from raw NIST data
- Introduced `Fr_features.csv` and `Na_features.csv` to include energy configurations and quantum numbers
- Added configurations for multiple electron states and levels with uncertainties
- Integrated support for Fr and Na isotopic datasets, expanding atomic dataset capabilities for energy modeling
</commit_message>
<xml_diff>
--- a/saved_models/results.xlsx
+++ b/saved_models/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PyCharmProjects\AtomEnergyLevels\saved_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B632F2-4FB9-4E05-95FF-ADD0C227CC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9A952D-1025-4817-A2EF-C99414EE4EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6870" yWindow="2310" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="K" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
   <si>
     <t>Mean Squared Error (MSE)</t>
   </si>
@@ -81,9 +81,6 @@
     <t>Binded, KDE</t>
   </si>
   <si>
-    <t>surface</t>
-  </si>
-  <si>
     <t>3867.19 cm⁻¹</t>
   </si>
   <si>
@@ -97,6 +94,9 @@
   </si>
   <si>
     <t xml:space="preserve"> 3867.19 cm⁻¹</t>
+  </si>
+  <si>
+    <t>13613092.00</t>
   </si>
 </sst>
 </file>
@@ -416,16 +416,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.1328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B1" t="s">
         <v>14</v>
       </c>
@@ -439,7 +439,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -450,13 +450,13 @@
         <v>14955167</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E2">
         <v>14955168</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -464,13 +464,16 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -478,13 +481,16 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -492,13 +498,16 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -508,11 +517,14 @@
       <c r="C6">
         <v>0.216</v>
       </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
       <c r="E6">
         <v>0.216</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -522,11 +534,14 @@
       <c r="C7" s="1">
         <v>9.6799999999999997E-2</v>
       </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
       <c r="E7" s="1">
         <v>9.6799999999999997E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -534,10 +549,13 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(AtomicDataset): add quantum defects and log target transformation
- Introduced quantum defects computation for potassium (K), including `n_star` and `rydberg_prediction`.
- Added support for logarithmic target transformations ('log-raw', 'log-binded', etc.).
- Updated target tagging logic and YAML configuration to enable `use_log_target`.
- Enhanced sample weighting options and tagging with consistent naming conventions.
</commit_message>
<xml_diff>
--- a/saved_models/results.xlsx
+++ b/saved_models/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PyCharmProjects\AtomEnergyLevels\saved_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC354A9-FB50-467F-BFBE-14D82775DC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8754FB15-EAC8-4B46-BEFA-ABCB3771466E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="13763" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="13763" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="K" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="71">
   <si>
     <t>Mean Squared Error (MSE)</t>
   </si>
@@ -233,7 +233,13 @@
     <t>binded, no weights</t>
   </si>
   <si>
-    <t>inversed binded, no weights</t>
+    <t>log binded, no weights</t>
+  </si>
+  <si>
+    <t>inversed raw, no weights</t>
+  </si>
+  <si>
+    <t>inversed binded (with clipping), no weights</t>
   </si>
 </sst>
 </file>
@@ -602,15 +608,6 @@
       <c r="B2">
         <v>13201036</v>
       </c>
-      <c r="C2">
-        <v>13201036</v>
-      </c>
-      <c r="D2">
-        <v>13201036</v>
-      </c>
-      <c r="E2">
-        <v>13201036</v>
-      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
@@ -619,15 +616,6 @@
       <c r="B3">
         <v>3633.32299804687</v>
       </c>
-      <c r="C3">
-        <v>3633.32299804687</v>
-      </c>
-      <c r="D3">
-        <v>3633.32299804687</v>
-      </c>
-      <c r="E3">
-        <v>3633.32299804687</v>
-      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
@@ -635,15 +623,6 @@
       </c>
       <c r="B4">
         <v>2027.59313964843</v>
-      </c>
-      <c r="C4">
-        <v>2027.59313964843</v>
-      </c>
-      <c r="D4">
-        <v>2027.59313964843</v>
-      </c>
-      <c r="E4">
-        <v>2027.59326171875</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
@@ -653,15 +632,6 @@
       <c r="B5">
         <v>1243.9453125</v>
       </c>
-      <c r="C5">
-        <v>1243.9453125</v>
-      </c>
-      <c r="D5">
-        <v>1243.9453125</v>
-      </c>
-      <c r="E5">
-        <v>1243.9453125</v>
-      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
@@ -670,15 +640,6 @@
       <c r="B6">
         <v>0.30797845125198298</v>
       </c>
-      <c r="C6">
-        <v>0.30797845125198298</v>
-      </c>
-      <c r="D6">
-        <v>0.30797845125198298</v>
-      </c>
-      <c r="E6">
-        <v>0.30797845125198298</v>
-      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
@@ -687,15 +648,6 @@
       <c r="B7">
         <v>9.1373691558837802</v>
       </c>
-      <c r="C7">
-        <v>9.1373691558837802</v>
-      </c>
-      <c r="D7">
-        <v>9.1373691558837802</v>
-      </c>
-      <c r="E7">
-        <v>9.1373691558837802</v>
-      </c>
       <c r="G7" s="1"/>
       <c r="I7" s="1"/>
     </row>
@@ -704,15 +656,6 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>16457.9375</v>
-      </c>
-      <c r="C8">
-        <v>16457.9375</v>
-      </c>
-      <c r="D8">
-        <v>16457.9375</v>
-      </c>
-      <c r="E8">
         <v>16457.9375</v>
       </c>
     </row>
@@ -2045,7 +1988,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA7832-422D-474D-9029-8C20BADED3EB}">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.3984375" bestFit="1" customWidth="1"/>
@@ -2477,7 +2420,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
@@ -2530,161 +2473,459 @@
       <c r="A28" t="s">
         <v>59</v>
       </c>
-      <c r="B28">
-        <v>20997686</v>
-      </c>
-      <c r="C28">
-        <v>20357744</v>
-      </c>
-      <c r="D28">
-        <v>16972888</v>
-      </c>
-      <c r="E28">
-        <v>18383196</v>
-      </c>
-      <c r="F28" s="4">
-        <v>4.0000000801635002E+20</v>
-      </c>
-      <c r="G28">
-        <v>20352586</v>
-      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>60</v>
       </c>
-      <c r="B29">
-        <v>4582.3232421875</v>
-      </c>
-      <c r="C29">
-        <v>4511.95556640625</v>
-      </c>
-      <c r="D29">
-        <v>4119.81640625</v>
-      </c>
-      <c r="E29">
-        <v>4287.56298828125</v>
-      </c>
-      <c r="F29">
-        <v>20000000000</v>
-      </c>
-      <c r="G29">
-        <v>4511.38427734375</v>
-      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>61</v>
       </c>
-      <c r="B30">
-        <v>1598.52185058593</v>
-      </c>
-      <c r="C30">
-        <v>1598.38427734375</v>
-      </c>
-      <c r="D30">
-        <v>1468.82458496093</v>
-      </c>
-      <c r="E30">
-        <v>1429.82641601562</v>
-      </c>
-      <c r="F30">
-        <v>4000001024</v>
-      </c>
-      <c r="G30">
-        <v>1566.6474609375</v>
-      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>62</v>
       </c>
-      <c r="B31">
-        <v>99.00390625</v>
-      </c>
-      <c r="C31">
-        <v>128.67578125</v>
-      </c>
-      <c r="D31">
-        <v>123.16796875</v>
-      </c>
-      <c r="E31">
-        <v>66.74609375</v>
-      </c>
-      <c r="F31">
-        <v>62.05078125</v>
-      </c>
-      <c r="G31">
-        <v>138.578125</v>
-      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>63</v>
       </c>
-      <c r="B32">
-        <v>-0.100734829902648</v>
-      </c>
-      <c r="C32">
-        <v>-6.7188024520873996E-2</v>
-      </c>
-      <c r="D32">
-        <v>0.110252022743225</v>
-      </c>
-      <c r="E32">
-        <v>3.63211631774902E-2</v>
-      </c>
-      <c r="F32">
-        <v>-20968688844800</v>
-      </c>
-      <c r="G32">
-        <v>-6.6917657852172796E-2</v>
-      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>64</v>
       </c>
-      <c r="B33">
-        <v>9.00884914398193</v>
-      </c>
-      <c r="C33">
-        <v>8.9274435043334908</v>
-      </c>
-      <c r="D33">
-        <v>8.1759958267211896</v>
-      </c>
-      <c r="E33">
-        <v>8.2598686218261701</v>
-      </c>
-      <c r="F33">
-        <v>13064511</v>
-      </c>
-      <c r="G33">
-        <v>8.8551073074340803</v>
-      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>65</v>
       </c>
-      <c r="B34">
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>57</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38">
+        <v>5</v>
+      </c>
+      <c r="F38">
+        <v>7</v>
+      </c>
+      <c r="G38">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>66</v>
+      </c>
+      <c r="B39">
+        <v>11137</v>
+      </c>
+      <c r="C39">
+        <v>11393</v>
+      </c>
+      <c r="D39">
+        <v>11649</v>
+      </c>
+      <c r="E39">
+        <v>12161</v>
+      </c>
+      <c r="F39">
+        <v>12673</v>
+      </c>
+      <c r="G39">
+        <v>13441</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>59</v>
+      </c>
+      <c r="B40">
+        <v>20997686</v>
+      </c>
+      <c r="C40">
+        <v>20357744</v>
+      </c>
+      <c r="D40">
+        <v>16972888</v>
+      </c>
+      <c r="E40">
+        <v>18383196</v>
+      </c>
+      <c r="F40" s="4">
+        <v>4.0000000801635002E+20</v>
+      </c>
+      <c r="G40">
+        <v>20352586</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>60</v>
+      </c>
+      <c r="B41">
+        <v>4582.3232421875</v>
+      </c>
+      <c r="C41">
+        <v>4511.95556640625</v>
+      </c>
+      <c r="D41">
+        <v>4119.81640625</v>
+      </c>
+      <c r="E41">
+        <v>4287.56298828125</v>
+      </c>
+      <c r="F41">
+        <v>20000000000</v>
+      </c>
+      <c r="G41">
+        <v>4511.38427734375</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>61</v>
+      </c>
+      <c r="B42">
+        <v>1598.52185058593</v>
+      </c>
+      <c r="C42">
+        <v>1598.38427734375</v>
+      </c>
+      <c r="D42">
+        <v>1468.82458496093</v>
+      </c>
+      <c r="E42">
+        <v>1429.82641601562</v>
+      </c>
+      <c r="F42">
+        <v>4000001024</v>
+      </c>
+      <c r="G42">
+        <v>1566.6474609375</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>62</v>
+      </c>
+      <c r="B43">
+        <v>99.00390625</v>
+      </c>
+      <c r="C43">
+        <v>128.67578125</v>
+      </c>
+      <c r="D43">
+        <v>123.16796875</v>
+      </c>
+      <c r="E43">
+        <v>66.74609375</v>
+      </c>
+      <c r="F43">
+        <v>62.05078125</v>
+      </c>
+      <c r="G43">
+        <v>138.578125</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44">
+        <v>-0.100734829902648</v>
+      </c>
+      <c r="C44">
+        <v>-6.7188024520873996E-2</v>
+      </c>
+      <c r="D44">
+        <v>0.110252022743225</v>
+      </c>
+      <c r="E44">
+        <v>3.63211631774902E-2</v>
+      </c>
+      <c r="F44">
+        <v>-20968688844800</v>
+      </c>
+      <c r="G44">
+        <v>-6.6917657852172796E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45">
+        <v>9.00884914398193</v>
+      </c>
+      <c r="C45">
+        <v>8.9274435043334908</v>
+      </c>
+      <c r="D45">
+        <v>8.1759958267211896</v>
+      </c>
+      <c r="E45">
+        <v>8.2598686218261701</v>
+      </c>
+      <c r="F45">
+        <v>13064511</v>
+      </c>
+      <c r="G45">
+        <v>8.8551073074340803</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>65</v>
+      </c>
+      <c r="B46">
         <v>21500.744140625</v>
       </c>
-      <c r="C34">
+      <c r="C46">
         <v>21045.197265625</v>
       </c>
-      <c r="D34">
+      <c r="D46">
         <v>19192.361328125</v>
       </c>
-      <c r="E34">
+      <c r="E46">
         <v>20329.900390625</v>
       </c>
-      <c r="F34">
+      <c r="F46">
         <v>99999997952</v>
       </c>
-      <c r="G34">
+      <c r="G46">
         <v>21227.021484375</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A49" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A50" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50">
+        <v>3</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>7</v>
+      </c>
+      <c r="G50">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51">
+        <v>11137</v>
+      </c>
+      <c r="C51">
+        <v>11393</v>
+      </c>
+      <c r="D51">
+        <v>11649</v>
+      </c>
+      <c r="E51">
+        <v>12161</v>
+      </c>
+      <c r="F51">
+        <v>12673</v>
+      </c>
+      <c r="G51">
+        <v>13441</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52">
+        <v>16448689</v>
+      </c>
+      <c r="C52">
+        <v>12672312</v>
+      </c>
+      <c r="D52">
+        <v>12114899</v>
+      </c>
+      <c r="E52">
+        <v>11117850</v>
+      </c>
+      <c r="F52">
+        <v>11424037</v>
+      </c>
+      <c r="G52">
+        <v>12324045</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53">
+        <v>4055.6982421875</v>
+      </c>
+      <c r="C53">
+        <v>3559.81909179687</v>
+      </c>
+      <c r="D53">
+        <v>3480.64624023437</v>
+      </c>
+      <c r="E53">
+        <v>3334.34399414062</v>
+      </c>
+      <c r="F53">
+        <v>3379.9462890625</v>
+      </c>
+      <c r="G53">
+        <v>3510.56201171875</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54">
+        <v>1314.94775390625</v>
+      </c>
+      <c r="C54">
+        <v>1083.91198730468</v>
+      </c>
+      <c r="D54">
+        <v>1063.09594726562</v>
+      </c>
+      <c r="E54">
+        <v>1005.49749755859</v>
+      </c>
+      <c r="F54">
+        <v>1029.32458496093</v>
+      </c>
+      <c r="G54">
+        <v>1072.7138671875</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55">
+        <v>206.48046875</v>
+      </c>
+      <c r="C55">
+        <v>137.33984375</v>
+      </c>
+      <c r="D55">
+        <v>109.01171875</v>
+      </c>
+      <c r="E55">
+        <v>101.171875</v>
+      </c>
+      <c r="F55">
+        <v>119.4453125</v>
+      </c>
+      <c r="G55">
+        <v>127.51953125</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A56" t="s">
+        <v>63</v>
+      </c>
+      <c r="B56">
+        <v>0.137731432914733</v>
+      </c>
+      <c r="C56">
+        <v>0.33569556474685602</v>
+      </c>
+      <c r="D56">
+        <v>0.36491608619689903</v>
+      </c>
+      <c r="E56">
+        <v>0.41718316078186002</v>
+      </c>
+      <c r="F56">
+        <v>0.40113228559494002</v>
+      </c>
+      <c r="G56">
+        <v>0.35395234823226901</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A57" t="s">
+        <v>64</v>
+      </c>
+      <c r="B57">
+        <v>7.7218508720397896</v>
+      </c>
+      <c r="C57">
+        <v>6.5894818305969203</v>
+      </c>
+      <c r="D57">
+        <v>6.4378457069396902</v>
+      </c>
+      <c r="E57">
+        <v>6.1210474967956499</v>
+      </c>
+      <c r="F57">
+        <v>6.2541313171386701</v>
+      </c>
+      <c r="G57">
+        <v>6.5000338554382298</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A58" t="s">
+        <v>65</v>
+      </c>
+      <c r="B58">
+        <v>19503.509765625</v>
+      </c>
+      <c r="C58">
+        <v>17312.58984375</v>
+      </c>
+      <c r="D58">
+        <v>16905.634765625</v>
+      </c>
+      <c r="E58">
+        <v>16195.60546875</v>
+      </c>
+      <c r="F58">
+        <v>16387.603515625</v>
+      </c>
+      <c r="G58">
+        <v>17043.69140625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>